<commit_message>
docs(qp): RTLabs/Gosuslugi PM interview cheat sheet from resume
Rebuild multi-sheet xlsx for Pavel Bidzhiev → RTLabs Project Manager
(Max voice assistant + contact-center support teams), mapped to Beeline
Problem Management and delivery metrics.

Co-authored-by: pagasbot-coder <pagasbot-coder@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/quiet-partner/docs/interview-pm-cheat-sheet.xlsx
+++ b/quiet-partner/docs/interview-pm-cheat-sheet.xlsx
@@ -9,12 +9,14 @@
   <sheets>
     <sheet name="Навигация" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Легенда" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Кейсы" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Exolve" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ХардСофт" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Словарик" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Вопросы" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Посмотреть" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Вакансия" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2 команды" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Кейсы" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Цифры Beeline" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ХардСофт" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Словарик" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Вопросы" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Посмотреть" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,7 +42,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,18 +72,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -444,12 +448,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,109 +486,269 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Старт собеса, «расскажите о себе»</t>
+          <t>Старт: «расскажите о себе»</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Кейсы</t>
+          <t>Вакансия</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ответы на типовые вопросы PM</t>
+          <t>Что ждут + твой мэппинг 1:1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Тех/поведенческое интервью</t>
+          <t>До собеса и перед кейсами</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Exolve</t>
+          <t>2 команды</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Доп. блок под МТС Exolve / антифрод</t>
+          <t>Макс (ИИ) + поддержка КЦ — как вести обе</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Если вакансия compliance / telecom</t>
+          <t>«Как будете вести 2 команды»</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ХардСофт</t>
+          <t>Кейсы</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hard + soft skills</t>
+          <t>Типовые вопросы PM + ответы на твоём опыте</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>«Чем сильнее слабее»</t>
+          <t>Тех / поведенческое</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Словарик</t>
+          <t>Цифры Beeline</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Термины одной строкой</t>
+          <t>Метрики одним взглядом</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Telecom / compliance</t>
+          <t>Когда просят цифры</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Вопросы</t>
+          <t>ХардСофт</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Что спросить у них</t>
+          <t>Hard + soft + Jira/Confluence</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>«Ваши вопросы?»</t>
+          <t>«Чем сильнее / слабее»</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Словарик</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Госуслуги / Макс / Agile</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Не путаться в терминах</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Вопросы</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Что спросить у них</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Конец интервью</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Посмотреть</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ссылки Habr / RTLabs + чеклист дня</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Домашняя подготовка</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Что</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ссылка / заметка</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Habr: как устроен Макс</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://habr.com/ru/companies/rtlabs/articles/587034/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Habr: Макс + LLM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://habr.com/ru/companies/rtlabs/articles/884694/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>One Day Offer / Робот Макс</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://about.rtlabs.ru/onedayoffer/robotmaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Кейс LLM / точность</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://generation-ai.ru/cases/gosuslugi-robot-maks</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Портал</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.gosuslugi.ru/ — потрогать Макса руками до собеса</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Референс формата шпаргалки</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2rfo3Q9ie1c</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>День до собеса</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ссылки и напоминания</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Подготовка дома</t>
+          <t>1) Intro 90 сек вслух 3 раза 2) лист «2 команды» 3) 5 вопросов 4) 5 цифр Beeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Не обещать</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Внутренние % РТЛабс без их данных; «я уже вёл Макса»; сроки без оценки команды</t>
         </is>
       </c>
     </row>
@@ -599,8 +763,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -613,7 +777,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Самопрезентация</t>
+          <t>Самопрезентация — Павел Биджиев · PM / PO · РТЛабс</t>
         </is>
       </c>
     </row>
@@ -625,12 +789,12 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Какой проект (последний / целевой)</t>
+          <t>Последний проект (Beeline)</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Состав команды (типовой)</t>
+          <t>Состав команды (Beeline)</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -640,44 +804,44 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Почему ищешь новое</t>
+          <t>Почему ищу новое / РТЛабс</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>Что ищешь сейчас (из вакансии)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Что ищу сейчас (из вакансии)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="120" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Госконтур (КБПК, администрация Кириш), ритейл («Твоя цена», контроль/СБ), потом IT: телеком, EdTech, PM-инструменты. Перешёл в PM ради измеримого результата и управления сроками/рисками.</t>
+          <t>Госконтур: директор МП КБПК ~3 г 5 мес; замглавы Кириши ~1 г — бюджет, 44-ФЗ, органы. Ритейл «Твоя цена» 3 г 8 мес, штат 73, логистика Китай→РФ. В IT с 2018: BA → PM/PO. Ценю измеримый delivery и ответственность за срок/качество.</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Целевой: МТС Exolve — compliance антифрод + ГИС «Антифрод». Параллельно: ProductMap (EdTech, PM frameworks). Beeline: интеграции, Problem Management, observability доступности с 23% до 97%.</t>
+          <t>Билайн с авг 2024: PO / рук. направления. ЛК B2B/B2C фикс+моб, highload 40+ млн аккаунтов, 6+ млн запросов/день, 10+ систем. Миграция ЦОД. Problem Management. E2E observability. AI: Cursor, NotebookLM.</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>PM + продукт + юристы + ИБ + DevOps + разработка + сеть/телефония + support. На Exolve — уточнить на собесе фактический состав.</t>
+          <t>Команда ~10. Кросс-стрим, корп. архитектура по 4 продуктам. Гибрид: Scrum (фичи) + Kanban (техдолг/инциденты). Бэклог 300+ задач. Roadmap Confluence↔Jira. Гант: зависимости Story/Sub-task → согласование планов −40%.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Сроки под регуляторику и НПА, реестр обязательств, gap по продуктам, риски, релизы, статус стейкхолдерам, интеграции, runbook до go-live.</t>
+          <t>Delivery и roadmap; бюджет продукта; приоритеты бэклога; Problem Management; мониторинг/SLA; согласование с архитектурой; статус стейкхолдерам; качество релизов.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>[ЗАПОЛНИ под вакансию: 1 факт + 1 цель, без негатива]</t>
+          <t>HR-этап пройден. РТЛабс — Госуслуги, соцзначимый масштаб, delivery в Agile/SAFe. Близко: highload, поддержка, автоматизация, ИИ-ассистент. Формат: офис/гибрид, Москва/СПб ок.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Проект с жёсткими дедлайнами закона, где PM ведёт план-график и метрики соответствия; влияние на бизнес (FP, SLA ГИС), не «ML ради ML».</t>
+          <t>PM: дейли/планирование/ревью/груминг/ретро; delivery по roadmap; 2 команды (Макс + КЦ); смежные; процессы; отчётность; актуальная документация; риски без сюрпризов.</t>
         </is>
       </c>
     </row>
@@ -690,9 +854,9 @@
       <c r="F4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Intro 60–90 сек (выучить)</t>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Intro 60–90 сек (выучить вслух)</t>
         </is>
       </c>
       <c r="B5" s="3" t="n"/>
@@ -701,10 +865,10 @@
       <c r="E5" s="3" t="n"/>
       <c r="F5" s="3" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>PM с опытом интеграций, рисков и дедлайнов в телекоме и госконтуре. На Exolve вижу проект compliance + ГИС «Антифрод»: реестр НПА → gap по продуктам → план под даты регулятора → интеграции и ops → метрики ложных блокировок для B2B. СОРМ и антифрод не смешиваю. Прямых переговоров с РКН и своего antifraud engine не строил — близко Beeline (интеграции, сроки, observability 23→97%) и работа с НПА в госконтуре.</t>
+          <t>Павел Биджиев, PM/PO. Сейчас в билайне веду направление ЛК: highload, команда ~10, Scrum+Kanban, бэклог 300+, roadmap в Confluence/Jira. Цифры: observability 23→97%, FRT инцидентов 3 ч→20 мин, Problem Management (повторяемость −35%, закрытие 14→5 дней), TTM −30%. До IT — госконтур и операционка: дедлайны, НПА, штат. На РТЛабс вижу роль PM по delivery двух контуров автоматизации поддержки Госуслуг: голосовой/цифровой ассистент Макс (ИИ) и команда КЦ (тикиты, баги, доработки). Мой фокус — ритм Agile, сроки/качество релизов, координация смежных, прозрачный статус и риски.</t>
         </is>
       </c>
       <c r="B6" s="3" t="n"/>
@@ -729,10 +893,18 @@
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A6:F8"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A6:F9"/>
     <mergeCell ref="A5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -745,166 +917,266 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Вопрос</t>
+          <t>Требование / обязанность РТЛабс</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ответ</t>
+          <t>Доказательство из опыта</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Что сказать одной фразой</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Нет документации на проекте</t>
+          <t>Дейли, планирование, обзор, груминг, ретро</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Привлечь системного аналитика или бывшего сотрудника для интервью. Параллельно правило: новая фича/интеграция → артефакт в wiki до релиза. Кontрольные точки у PM: что, кто, когда. Не завязать знания на одном человеке.</t>
+          <t>Beeline: гибрид Scrum+Kanban, регулярные церемонии, roadmap</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Ритм команды держу сам: планирование фич + поток инцидентов/техдолга отдельно.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Уходит главный / ключевой разработчик</t>
+          <t>Координация дизайнеров, аналитиков, dev, QA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>1-on-1: сценарий «остаётся / уходит». Если уходит — описание архитектуры, handover 1–1,5 мес, сразу найм, подключить соседний юнит. Профилактика: bus factor в реестре рисков с первого месяца.</t>
+          <t>Команда ~10 + кросс-стрим + корп. архитектура 4 продукта</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Свожу роли в один план: зависимости в Ганте, приоритеты в Jira.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Техдолг — как приоритизируешь</t>
+          <t>Delivery: релизы, сроки, качество, roadmap</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Блокер релиза &gt; влияние на KPI/фичи &gt; быстрые wins. Окно между релизами или конец года. Compliance must-have — отдельная очередь, не «удобный рефакторинг».</t>
+          <t>TTM 6→4 нед (−30%); баги/техтребования −15%; миграция ЦОД</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Отвечаю за поставку по карте релизов, не только за «провести митинг».</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Инцидент в пятницу вечером</t>
+          <t>Смежные / внешние команды</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Сначала стабилизация: runbook, дежурный, эскалация. Потом retro — почему и как не повторить. Для ГИС отдельно: SLA 24/7, RTO/RPO (уточнить у Exolve).</t>
+          <t>Архитектура, стрим, 10+ интеграций ЛК</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Технические и оргвопросы закрываю через явных владельцев и эскалацию по SLA.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Inhouse vs аутстаф / аутсорс</t>
+          <t>Улучшение процессов</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Inhouse: погружение, скорость изменений, дороже, хуже масштаб. Аутстаф: гибко и дешевле, нужны контрольные точки. Ответственность перед регулятором не делегирую «на подрядчика без RACI».</t>
+          <t>Problem Management; observability; согласование планов −40%</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Сначала метрика боли, потом процесс: инциденты → корневые причины → playbook.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Проблема, которую никто не может решить</t>
+          <t>Отчётность по направлениям</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Декомпозиция → аналоги → эксперты внутри/снаружи → гипотезы → решение. С бизнесом — язык денег: критичность vs стоимость поиска (как с диагностикой авто).</t>
+          <t>Единая страница roadmap Confluence↔Jira; статус стейкхолдерам</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Один экран: план / факт / риски / решения — без сюрприза в конце спринта.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Была документация на проекте?</t>
+          <t>Актуальная проектная документация</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Устав, ТЗ/ФТ, user stories, реестр рисков, runbook. На compliance — реестр НПА как single source of truth. PM/Legal следят за актуальностью.</t>
+          <t>Confluence roadmap; база известных ошибок L2; диаграмма развёртывания</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Документация = рабочий артефакт для команды, не «отчёт ради отчёта».</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Онбординг разработчика без документации</t>
+          <t>Несколько направлений: масштаб, фичи, каналы, пользователи</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Intro → доступы → чаты → buddy → мелкие задачи → фиксировать находки в wiki с day 1. Параллельно процесс обязательной документации.</t>
+          <t>ЛК WEB + non-WEB; 4 продукта; ProductMap AI/ML; ЦЕНТРОФИНАНС лояльность</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Привык вести параллельные потоки с общим приоритетом и общим статусом.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Спор разработчиков (стек / Python vs Go)</t>
+          <t>Информирование о прогрессе, изменениях, рисках</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Синки 1-on-1 → общий митинг, медиатор. Язык цифр: скорость MVP, поддержка, масштаб. Решение в ADR. Для MVP — что быстрее к ценности; для платформы — что жить 3+ года.</t>
+          <t>Реестр рисков; Problem Management; статус без сюрпризов</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Риск поднимаю рано, с владельцем и датой решения.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>От кого задачи / стейкхолдеры</t>
+          <t>PO/PM от 2 лет, Agile Scrum/Kanban</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Спонсор, продукт, юристы, ИБ, CTO/архитектор, ops, support. На Exolve: кто A по сроку регулятора — имя, не «отдел».</t>
+          <t>Beeline 2+ г; ProductMap 2 г 10 мес; MEXC 2 г 3 мес</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>И delivery, и product-бэклог — умею оба режима.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Прямые подчинённые?</t>
+          <t>Jira/Confluence: доски, фильтры, dashboards</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Честно: в Scrum часто без formal line, но delivery, приоритеты, риски, статус — на PM. RACI вместо «все подчинены мне».</t>
+          <t>Roadmap Confluence + Jira; сегментация бэклога 300+; High/Med/Low + вес</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Доски и дашборды настраиваю под delivery, не «красивую картинку».</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Когда документируешь задачу</t>
+          <t>Цикл разработки ПО, язык с разработчиками</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Discovery → Delivery: user story, критерии приёмки, задачи. Системная аналитика/API — до кода. Confluence — до merge для новых интеграций.</t>
+          <t>Highload, интеграции, миграция ЦОД, AI Cursor</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Не пишу код за команду, но понимаю зависимости, риски релиза и DoD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Приоритизация MoSCoW / RICE / Value-Effort</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>High/Med/Low + вес; Value/Effort на ProductMap и ЦЕНТРОФИНАНС</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Приоритет = влияние на метрику × стоимость × риск регулятора/SLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Офис / гибрид, 5/2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Москва, готов СПб, командировки</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Формат работодателя ок; готов к гибриду на месте.</t>
         </is>
       </c>
     </row>
@@ -919,11 +1191,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -934,91 +1207,148 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ответ / факт</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>Команда 1 — Робот Макс (ИИ / голос)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Команда 2 — Поддержка КЦ (тикиты / баги)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="70" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Суть Exolve</t>
+          <t>Что это (публично)</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Голос, SMS, API, 8-800, B2B. Антифрод = compliance + продукт + бизнес.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Цифровой ассистент Госуслуг: веб, приложение, голос. LLM (в т.ч. YandexGPT), консультации, поиск услуг. Публично: большой DAU, высокая автоматизация ответов, фокус на точности и latency.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Контур контакт-центра: тикеты, баги, доработки системы поддержки. Снижение очереди к оператору, качество ответов, стабильность инструментов КЦ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="70" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>СОРМ ≠ антифрод</t>
+          <t>Моя роль PM</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>СОРМ: 126+144 ФЗ, доступ органов. Антифрод: ГИС, сигналы, блокировки, маркировка.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Delivery фич Макса: релизы, качество ответов/голос, координация ML/аналитики/dev/QA, риски галлюцинаций и эскалации на человека.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Delivery бэклога поддержки: баги, улучшения, SLA тикетов, связь с L1/L2, база знаний, Problem Management.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="70" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Подход PM</t>
+          <t>Метрики (спросить у них / предложить)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Реестр НПА → gap matrix → план под даты → интеграции + ops → FP rate для B2B.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Автоматизация %, CSAT/дизлайки ответов, containment (без оператора), latency голоса, accuracy / эскалация в человека, coverage сценариев.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>FRT, MTTR, повторные обращения, % тикетов без эскалации, CSAT КЦ, backlog aging, escape defects в прод.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="70" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>90 дней (каркас)</t>
+          <t>Мой мост из Beeline</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>1–30: реестр, gap, RACI. 31–60: MVP интеграции, пилот. 61–90: scope, автоматизация, аудит.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>AI-инструменты + продуктовый AI/ML (ProductMap); highload и интеграции; качество «ответа» пользователю.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Problem Management: повторяемость −35%, FRT 3ч→20м, проактив 10→40%, закрытие проблем 14→5 дн; observability 23→97%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Честные пробелы</t>
+          <t>Как веду обе сразу</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Нет прямых переговоров с РКН; нет deep СОРМ; не строил antifraud engine оператора.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>Два бэклога, один ритм статуса. Общий weekly: зависимости Макс↔КЦ (эскалация, база знаний, голос→тикет).</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Kanban для инцидентов/багов КЦ + Scrum-спринты для фич Макса. Общий риск-реестр и единый статус спонсору.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Не обещать</t>
+          <t>Риски</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Даты НПА из СМИ; «уже построил ГИС»; смешение СОРМ и антифрода в одном эпике.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Неточные ответы ИИ на госуслугах; задержка голоса; изменение НПА/услуг → устаревшая база знаний.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Очередь тикетов; выгорание; баги тулов КЦ; bus factor; нет документации сценариев.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>KPI проекта</t>
+          <t>Первые 30 дней</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Coverage к дате N; 0 критичных предписаний; SLA ГИС; FP ≤ X%; time-to-block/report.</t>
+          <t>Карта стейкхолдеров Макса; текущие KPI; DoD релиза; процесс эскалации в человека; что в roadmap квартала.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Карта потока тикета; SLA; топ-повторяющиеся причины; кто L2; что уже в Problem/Known Error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Не выдумывать на собесе</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Не обещать «я уже делал Макса». Сказать: публичный контекст знаю (Habr RTLabs), детали контура уточню у команды.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Не путать Макса (ассистент) и отдельный продукт «голосовой помощник» без уточнения у интервьюера.</t>
         </is>
       </c>
     </row>
@@ -1033,82 +1363,214 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="78" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Категория</t>
+          <t>Вопрос</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Содержание</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>Ответ (каркас под РТЛабс + мой опыт)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="55" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Hard — инструменты</t>
+          <t>Расскажите о себе / почему PM</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Jira, Confluence, Miro/Notion, статус-шаблон, диаграмма Ганта, реестр рисков.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Intro с Легенды. Акцент: delivery + метрики поддержки/highload + госконтур как понимание масштаба Госуслуг.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="55" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Hard — техника (уровень PM)</t>
+          <t>Как ведёте 2 команды параллельно</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>API/BFF, интеграции, observability, базово Docker/PostgreSQL. Не притворяться архитектором СОРМ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Два бэклога, общий статус. Scrum для фич Макса, Kanban для потока КЦ. Weekly синк зависимостей. Один риск-реестр. Не смешиваю WIP без приоритета спонсора.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Hard — сильная сторона</t>
+          <t>Нет документации</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Beeline: observability доступности 23% → 97%; интеграции; Problem Management.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Сразу процесс: новая фича/багфикс → артефакт в Confluence. Buddy + фиксация находок. Для КЦ — known error DB (как в Problem Management). Контрольные точки у PM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Soft</t>
+          <t>Уходит ключевой разработчик</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Медиатор, язык цифр, честные пробелы, 1-on-1, статус без сюрпризов, работа с юристами.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>1-on-1: остаётся / уходит. Если уходит — архитектура + handover 1–1,5 мес + найм. Bus factor в рисках заранее. На госконтуре особенно критично.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Anti-patterns</t>
+          <t>Техдолг</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Блеф по НПА; обещания без юриста; scope creep без change control.</t>
+          <t>Не мёртвый груз: приоритет по блокеру релиза и влиянию на SLA/метрики. У меня: техдолг −30%. Окно между релизами. Must для стабильности КЦ/Макса не тонет в «удобном рефакторинге».</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Инцидент вечером / пятница</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Стабилизация по runbook → коммуникация → retro. В Beeline: FRT и observability. Для Госуслуг — эскалация и статус без паники, с владельцем.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Problem Management — что делали</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Повторяемость −35%; среднее решение −25%; проактив 10→40%; закрытие 14→5 дней. База известных ошибок + обучение L2. Прямой мост к команде КЦ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Как измерите успех автоматизации поддержки</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Containment/автоматизация %, CSAT, FRT/MTTR, повторные обращения, % эскалаций Макс→человек, качество ответов (дизлайки). Цифры целевые — согласую с владельцем продукта.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Спор разработчиков о стеке / подходе</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>1-on-1 → общая встреча, медиатор. Язык цифр: скорость, риск, поддержка, соответствие стеку платформы. Решение в ADR/Confluence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Inhouse vs подряд</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Inhouse: погружение. Подряд: масштаб. На Госуслугах ответственность за качество сервиса не «списать на подрядчика» — нужен RACI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="55" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Онбординг без документации</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Intro, доступы, чаты, buddy, мелкие задачи, писать wiki с day 1. Параллельно закрывать дыры в Confluence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="55" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Приоритизация (RICE / MoSCoW)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Value/Effort + риск SLA. Must для стабильности КЦ и критичных сценариев Макса. Should — рост автоматизации. Won't — без владельца метрики.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Конфликт приоритетов двух команд</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Эскалация спонсору с цифрами: влияние на пользователей Госуслуг / очередь КЦ. Фиксирую решение и пересбор roadmap на неделю.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="55" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Слабые стороны / пробелы</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Честно: не работал внутри команды Макса. Сильная сторона — highload support/observability и Problem Management. Детали контура Госуслуг уточню в первые 2 недели.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="55" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Почему РТЛабс / Госуслуги</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Соцзначимый масштаб, delivery в зрелом Agile/SAFe, автоматизация поддержки + ИИ. Близко к моему профилю: метрики сервиса, процессы, координация.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Как работаете с SAFe / несколькими поездами</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>На уровне команды — Scrum/Kanban. На уровне программы — единый статус, зависимости, риски. Уточню, как у вас нарезаны ART/поезда для Макса и КЦ.</t>
         </is>
       </c>
     </row>
@@ -1123,142 +1585,283 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Термин</t>
+          <t>Метрика</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Одна строка</t>
+          <t>Было → Стало</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Зачем на собесе РТЛабс</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>ГИС «Антифрод»</t>
+          <t>Observability доступности (3 продукта)</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Госсистема обмена сигналами; не путать с СОРМ</t>
+          <t>23% → 97%</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Надёжность сервиса / мониторинг — язык Госуслуг</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>СОРМ</t>
+          <t>FRT по инцидентам</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>126+144 ФЗ — доступ уполномоченных органов</t>
+          <t>3 часа → 20 минут</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Прямой мост к КЦ и SLA поддержки</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>FP / FN</t>
+          <t>Таймауты у потребителей</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Ложная блокировка / пропуск фрода</t>
+          <t>−75% (в 4 раза)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Качество интеграций / UX</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>ВАТС</t>
+          <t>Повторяемость инцидентов (Problem Mgmt)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Облачная телефония — отдельный legal + product impact</t>
+          <t>−35%</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Команда КЦ: меньше одних и тех же тикетов</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Gap matrix</t>
+          <t>Среднее время решения проблемы</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Требование → продукт Exolve → статус</t>
+          <t>−25%</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Known error + L2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Must / should</t>
+          <t>Проактивные решения</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Из реестра юриста, не из головы PM</t>
+          <t>10% → 40%</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Не только «тушить», а предотвращать</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>RACI</t>
+          <t>Время закрытия проблем</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>R исполнитель, A ответственный за результат, C консультант, I в курсе</t>
+          <t>14 → 5 дней</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Дисциплина Problem Management</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Runbook</t>
+          <t>CSAT поддержки</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Ops после go-live: дежурства, эскалации, RCA</t>
+          <t>+20%</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Чат-бот + обратная связь — рядом с Максом</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Time-to-block</t>
+          <t>Time-to-market</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Скорость блокировки по сигналу</t>
+          <t>6 → 4 недели (−30%)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Delivery / roadmap</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Rolling wave</t>
+          <t>Техдолг</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Детальный план на 2–3 недели, дальше — полосы</t>
+          <t>−30%</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Стабильность платформы</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Согласование планов</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>−40%</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Гант + зависимости — координация смежных</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Масштаб ЛК</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>40+ млн акк., 6+ млн req/day</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Готовность к высоконагруженным сервисам</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ProductMap</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>25k+ users, DAU 1760, LTV +15%</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Product mindset + AI/ML модуль</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ЦЕНТРОФИНАНС</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>NPS +15%, churn −5%</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Метрики удержания</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>MEXC кабинет партнёра</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>NPS промоутеров +21%, ER +26%</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>UX кабинета / дашборды</t>
         </is>
       </c>
     </row>
@@ -1273,102 +1876,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Категория</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Вопрос интервьюеру</t>
+          <t>Содержание</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Какая роль Exolve: оператор / агрегатор / партнёр МТС?</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Hard — Jira/Confluence</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Доски Scrum/Kanban, фильтры, dashboards, roadmap страница, связь эпик→story→sub-task, Гант.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Какие продукты in scope первой волны: API, SMS, голос, 8-800, ВАТС?</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Hard — delivery</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Roadmap/релизный план, DoD, зависимости смежных, статус, риски, отчётность.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Кто accountable за дедлайн регулятора — конкретное имя?</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Hard — support/ops</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Problem Management, known errors, SLA/FRT/MTTR, observability, эскалации.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Узел обмена с ГИС: SLA 24/7, RTO/RPO?</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Hard — product</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Бэклог, RICE/Value-Effort, CJM, custdev, unit-экономика (ProductMap, ЦЕНТРОФИНАНС).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Есть ли бюджет false positive для B2B (порог X%)?</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Hard — AI (честно)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Cursor/NotebookLM в работе; ProductMap AI/ML модуль. Макса изнутри не строил — быстро вхожу в контур.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Процесс апелляций / whitelist для легальных клиентов?</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Soft</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Медиатор, язык цифр, 1-on-1, статус без сюрпризов, работа с архитектурой и бизнесом.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Что уже сделано vs gap на старте?</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Госконтур</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>КБПК, администрация Кириши: дедлайны, НПА, стейкхолдеры, ответственность за результат.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Как устроена связка PM — Legal — ИБ — DevOps?</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Формат</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Москва; готов СПб; офис/гибрид; командировки; полный день 5/2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Языки</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Русский родной; English B2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Anti-patterns</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Не блефовать про Макса; не обещать % автоматизации без baseline; не тонуть в митингах без delivery.</t>
         </is>
       </c>
     </row>
@@ -1383,82 +2026,308 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Что</t>
+          <t>Термин</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ссылка / заметка</t>
+          <t>Одна строка</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Видео-референс шпаргалки</t>
-        </is>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>РТЛабс</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Техпартнёр цифровых сервисов Госуслуг; аккредитованная IT-компания</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Робот Макс</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Цифровой ассистент Госуслуг (чат/голос/приложение), в т.ч. LLM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Containment</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Доля обращений, закрытых без оператора</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>FRT</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>First Response Time — время первого ответа</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>MTTR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Mean Time To Resolve — среднее время решения</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Problem Management</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Работа с корневыми причинами, не только с инцидентами</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Known Error</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Известная ошибка с обходным путём / фиксом в базе</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>SAFe</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Масштабирование Agile на много команд — уточнить нарезку у них</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>ART</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Agile Release Train в SAFe</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>DoD</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Критерии готовности истории/релиза</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>MoSCoW / RICE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Фреймворки приоритизации</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Escalation to human</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Передача диалога Макса оператору КЦ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Наблюдаемость доступности/здоровья сервиса (у меня 23→97%)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Вопрос интервьюеру</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=2rfo3Q9ie1c</t>
+          <t>Как нарезаны 2 команды (Макс и КЦ): составы, PO/тимлиды, общий спонсор?</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Exolve prep (канон)</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>quiet-partner/knowledge-base/mts-exolve-antifraud-project-prep.md</t>
+          <t>Какие KPI успеха PM на испытательном: delivery, автоматизация, CSAT, FRT?</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Чеклист собеса</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>quiet-partner/docs/mts-exolve-next-checklist.md</t>
+          <t>Как устроен поток эскалации Макс → оператор → тикет в КЦ?</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Lifecycle playbook</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>quiet-partner/knowledge-base/project-lifecycle-playbook.md</t>
+          <t>Какой baseline автоматизации и где узкое место сейчас?</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Перед собесом</t>
-        </is>
+      <c r="A6" t="n">
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Проговорить intro 60–90 сек без бумаги; СОРМ ≠ антифрод одной фразой</t>
+          <t>Jira: одна доска на две команды или раздельные? Как видите зависимости?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SAFe: как часто PI-планирование и что от PM ждут на уровне поезда?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Кто A (accountable) за roadmap Макса и за бэклог КЦ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Какие смежные обязательны: ML, знание услуг, контакт-центр, безопасность?</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Формат: сколько дней в офисе, какой офис (Москва)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Что должно измениться через 90 дней, если найм успешен?</t>
         </is>
       </c>
     </row>

</xml_diff>